<commit_message>
feat(seo): optimize unified compact filter controls and sync live serp data 30/09/2026
</commit_message>
<xml_diff>
--- a/song_anh_seo_keywords_historical_database.xlsx
+++ b/song_anh_seo_keywords_historical_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1167"/>
+  <dimension ref="A1:I1233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45937,6 +45937,2580 @@
         </is>
       </c>
     </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1168" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>mô hình quy hoạch</t>
+        </is>
+      </c>
+      <c r="D1168" t="n">
+        <v>6</v>
+      </c>
+      <c r="E1168" t="n">
+        <v>80</v>
+      </c>
+      <c r="F1168" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1168" t="inlineStr">
+        <is>
+          <t>8.75%</t>
+        </is>
+      </c>
+      <c r="H1168" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I1168" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1169" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1169" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="E1169" t="n">
+        <v>323</v>
+      </c>
+      <c r="F1169" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1169" t="inlineStr">
+        <is>
+          <t>2.17%</t>
+        </is>
+      </c>
+      <c r="H1169" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1169" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1170" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>mô hình cao tầng</t>
+        </is>
+      </c>
+      <c r="D1170" t="n">
+        <v>5</v>
+      </c>
+      <c r="E1170" t="n">
+        <v>980</v>
+      </c>
+      <c r="F1170" t="n">
+        <v>54</v>
+      </c>
+      <c r="G1170" t="inlineStr">
+        <is>
+          <t>5.51%</t>
+        </is>
+      </c>
+      <c r="H1170" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I1170" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1171" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>mô hình nhà máy</t>
+        </is>
+      </c>
+      <c r="D1171" t="n">
+        <v>24</v>
+      </c>
+      <c r="E1171" t="n">
+        <v>29</v>
+      </c>
+      <c r="F1171" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1171" t="inlineStr">
+        <is>
+          <t>3.45%</t>
+        </is>
+      </c>
+      <c r="H1171" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
+        </is>
+      </c>
+      <c r="I1171" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1172" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>mô hình thiết bị</t>
+        </is>
+      </c>
+      <c r="D1172" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1172" t="n">
+        <v>640</v>
+      </c>
+      <c r="F1172" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1172" t="inlineStr">
+        <is>
+          <t>3.91%</t>
+        </is>
+      </c>
+      <c r="H1172" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
+        </is>
+      </c>
+      <c r="I1172" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1173" t="n">
+        <v>6</v>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>mô hình trường học</t>
+        </is>
+      </c>
+      <c r="D1173" t="n">
+        <v>7</v>
+      </c>
+      <c r="E1173" t="n">
+        <v>720</v>
+      </c>
+      <c r="F1173" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1173" t="inlineStr">
+        <is>
+          <t>5.28%</t>
+        </is>
+      </c>
+      <c r="H1173" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I1173" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1174" t="n">
+        <v>7</v>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>mô hình bệnh viện</t>
+        </is>
+      </c>
+      <c r="D1174" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1174" t="n">
+        <v>530</v>
+      </c>
+      <c r="F1174" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1174" t="inlineStr">
+        <is>
+          <t>4.15%</t>
+        </is>
+      </c>
+      <c r="H1174" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I1174" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1175" t="n">
+        <v>8</v>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>sa bàn quy hoạch</t>
+        </is>
+      </c>
+      <c r="D1175" t="n">
+        <v>4</v>
+      </c>
+      <c r="E1175" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F1175" t="n">
+        <v>118</v>
+      </c>
+      <c r="G1175" t="inlineStr">
+        <is>
+          <t>7.15%</t>
+        </is>
+      </c>
+      <c r="H1175" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I1175" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1176" t="n">
+        <v>9</v>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1176" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="E1176" t="n">
+        <v>43</v>
+      </c>
+      <c r="F1176" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1176" t="inlineStr">
+        <is>
+          <t>2.33%</t>
+        </is>
+      </c>
+      <c r="H1176" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1176" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1177" t="n">
+        <v>10</v>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>sa bàn cao tầng</t>
+        </is>
+      </c>
+      <c r="D1177" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E1177" t="n">
+        <v>870</v>
+      </c>
+      <c r="F1177" t="n">
+        <v>46</v>
+      </c>
+      <c r="G1177" t="inlineStr">
+        <is>
+          <t>5.29%</t>
+        </is>
+      </c>
+      <c r="H1177" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I1177" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1178" t="n">
+        <v>11</v>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>sa bàn nhà máy</t>
+        </is>
+      </c>
+      <c r="D1178" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E1178" t="n">
+        <v>28</v>
+      </c>
+      <c r="F1178" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1178" t="inlineStr">
+        <is>
+          <t>3.57%</t>
+        </is>
+      </c>
+      <c r="H1178" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
+        </is>
+      </c>
+      <c r="I1178" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1179" t="n">
+        <v>12</v>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>sa bàn thiết bị</t>
+        </is>
+      </c>
+      <c r="D1179" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E1179" t="n">
+        <v>480</v>
+      </c>
+      <c r="F1179" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1179" t="inlineStr">
+        <is>
+          <t>3.75%</t>
+        </is>
+      </c>
+      <c r="H1179" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
+        </is>
+      </c>
+      <c r="I1179" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1180" t="n">
+        <v>13</v>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>sa bàn trường học</t>
+        </is>
+      </c>
+      <c r="D1180" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="E1180" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1180" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1180" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="H1180" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I1180" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1181" t="n">
+        <v>14</v>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>sa bàn bệnh viện</t>
+        </is>
+      </c>
+      <c r="D1181" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E1181" t="n">
+        <v>590</v>
+      </c>
+      <c r="F1181" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1181" t="inlineStr">
+        <is>
+          <t>4.41%</t>
+        </is>
+      </c>
+      <c r="H1181" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
+        </is>
+      </c>
+      <c r="I1181" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1182" t="n">
+        <v>15</v>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>vận chuyển mô hình</t>
+        </is>
+      </c>
+      <c r="D1182" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E1182" t="n">
+        <v>820</v>
+      </c>
+      <c r="F1182" t="n">
+        <v>45</v>
+      </c>
+      <c r="G1182" t="inlineStr">
+        <is>
+          <t>5.49%</t>
+        </is>
+      </c>
+      <c r="H1182" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1182" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1183" t="n">
+        <v>16</v>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>vận chuyển sa bàn</t>
+        </is>
+      </c>
+      <c r="D1183" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E1183" t="n">
+        <v>760</v>
+      </c>
+      <c r="F1183" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1183" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="H1183" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1183" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1184" t="n">
+        <v>17</v>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>sửa chữa mô hình</t>
+        </is>
+      </c>
+      <c r="D1184" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E1184" t="n">
+        <v>930</v>
+      </c>
+      <c r="F1184" t="n">
+        <v>58</v>
+      </c>
+      <c r="G1184" t="inlineStr">
+        <is>
+          <t>6.24%</t>
+        </is>
+      </c>
+      <c r="H1184" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1184" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1185" t="n">
+        <v>18</v>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>sửa chữa sa bàn</t>
+        </is>
+      </c>
+      <c r="D1185" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E1185" t="n">
+        <v>880</v>
+      </c>
+      <c r="F1185" t="n">
+        <v>52</v>
+      </c>
+      <c r="G1185" t="inlineStr">
+        <is>
+          <t>5.91%</t>
+        </is>
+      </c>
+      <c r="H1185" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1185" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1186" t="n">
+        <v>19</v>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>công ty mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1186" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="E1186" t="n">
+        <v>69</v>
+      </c>
+      <c r="F1186" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1186" t="inlineStr">
+        <is>
+          <t>2.90%</t>
+        </is>
+      </c>
+      <c r="H1186" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="I1186" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1187" t="n">
+        <v>20</v>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>công ty sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1187" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E1187" t="n">
+        <v>2410</v>
+      </c>
+      <c r="F1187" t="n">
+        <v>168</v>
+      </c>
+      <c r="G1187" t="inlineStr">
+        <is>
+          <t>6.97%</t>
+        </is>
+      </c>
+      <c r="H1187" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/</t>
+        </is>
+      </c>
+      <c r="I1187" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1188" t="n">
+        <v>21</v>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>làm mô hình</t>
+        </is>
+      </c>
+      <c r="D1188" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E1188" t="n">
+        <v>1780</v>
+      </c>
+      <c r="F1188" t="n">
+        <v>121</v>
+      </c>
+      <c r="G1188" t="inlineStr">
+        <is>
+          <t>6.80%</t>
+        </is>
+      </c>
+      <c r="H1188" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1188" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B1189" t="n">
+        <v>22</v>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>làm sa bàn</t>
+        </is>
+      </c>
+      <c r="D1189" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E1189" t="n">
+        <v>1620</v>
+      </c>
+      <c r="F1189" t="n">
+        <v>104</v>
+      </c>
+      <c r="G1189" t="inlineStr">
+        <is>
+          <t>6.42%</t>
+        </is>
+      </c>
+      <c r="H1189" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I1189" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1190" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>mô hình quy hoạch</t>
+        </is>
+      </c>
+      <c r="D1190" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="E1190" t="n">
+        <v>82</v>
+      </c>
+      <c r="F1190" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1190" t="inlineStr">
+        <is>
+          <t>8.54%</t>
+        </is>
+      </c>
+      <c r="H1190" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I1190" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1191" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1191" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="E1191" t="n">
+        <v>338</v>
+      </c>
+      <c r="F1191" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1191" t="inlineStr">
+        <is>
+          <t>2.07%</t>
+        </is>
+      </c>
+      <c r="H1191" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1191" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1192" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>mô hình cao tầng</t>
+        </is>
+      </c>
+      <c r="D1192" t="n">
+        <v>5</v>
+      </c>
+      <c r="E1192" t="n">
+        <v>980</v>
+      </c>
+      <c r="F1192" t="n">
+        <v>54</v>
+      </c>
+      <c r="G1192" t="inlineStr">
+        <is>
+          <t>5.51%</t>
+        </is>
+      </c>
+      <c r="H1192" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I1192" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1193" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>mô hình nhà máy</t>
+        </is>
+      </c>
+      <c r="D1193" t="n">
+        <v>24</v>
+      </c>
+      <c r="E1193" t="n">
+        <v>29</v>
+      </c>
+      <c r="F1193" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1193" t="inlineStr">
+        <is>
+          <t>3.45%</t>
+        </is>
+      </c>
+      <c r="H1193" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
+        </is>
+      </c>
+      <c r="I1193" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1194" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>mô hình thiết bị</t>
+        </is>
+      </c>
+      <c r="D1194" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1194" t="n">
+        <v>640</v>
+      </c>
+      <c r="F1194" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1194" t="inlineStr">
+        <is>
+          <t>3.91%</t>
+        </is>
+      </c>
+      <c r="H1194" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
+        </is>
+      </c>
+      <c r="I1194" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1195" t="n">
+        <v>6</v>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>mô hình trường học</t>
+        </is>
+      </c>
+      <c r="D1195" t="n">
+        <v>7</v>
+      </c>
+      <c r="E1195" t="n">
+        <v>720</v>
+      </c>
+      <c r="F1195" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1195" t="inlineStr">
+        <is>
+          <t>5.28%</t>
+        </is>
+      </c>
+      <c r="H1195" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I1195" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1196" t="n">
+        <v>7</v>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>mô hình bệnh viện</t>
+        </is>
+      </c>
+      <c r="D1196" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1196" t="n">
+        <v>530</v>
+      </c>
+      <c r="F1196" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1196" t="inlineStr">
+        <is>
+          <t>4.15%</t>
+        </is>
+      </c>
+      <c r="H1196" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I1196" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1197" t="n">
+        <v>8</v>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>sa bàn quy hoạch</t>
+        </is>
+      </c>
+      <c r="D1197" t="n">
+        <v>4</v>
+      </c>
+      <c r="E1197" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F1197" t="n">
+        <v>118</v>
+      </c>
+      <c r="G1197" t="inlineStr">
+        <is>
+          <t>7.15%</t>
+        </is>
+      </c>
+      <c r="H1197" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I1197" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1198" t="n">
+        <v>9</v>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1198" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1198" t="n">
+        <v>44</v>
+      </c>
+      <c r="F1198" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1198" t="inlineStr">
+        <is>
+          <t>2.27%</t>
+        </is>
+      </c>
+      <c r="H1198" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1198" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1199" t="n">
+        <v>10</v>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>sa bàn cao tầng</t>
+        </is>
+      </c>
+      <c r="D1199" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E1199" t="n">
+        <v>870</v>
+      </c>
+      <c r="F1199" t="n">
+        <v>46</v>
+      </c>
+      <c r="G1199" t="inlineStr">
+        <is>
+          <t>5.29%</t>
+        </is>
+      </c>
+      <c r="H1199" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I1199" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1200" t="n">
+        <v>11</v>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>sa bàn nhà máy</t>
+        </is>
+      </c>
+      <c r="D1200" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E1200" t="n">
+        <v>28</v>
+      </c>
+      <c r="F1200" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1200" t="inlineStr">
+        <is>
+          <t>3.57%</t>
+        </is>
+      </c>
+      <c r="H1200" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
+        </is>
+      </c>
+      <c r="I1200" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1201" t="n">
+        <v>12</v>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>sa bàn thiết bị</t>
+        </is>
+      </c>
+      <c r="D1201" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E1201" t="n">
+        <v>480</v>
+      </c>
+      <c r="F1201" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1201" t="inlineStr">
+        <is>
+          <t>3.75%</t>
+        </is>
+      </c>
+      <c r="H1201" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
+        </is>
+      </c>
+      <c r="I1201" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1202" t="n">
+        <v>13</v>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>sa bàn trường học</t>
+        </is>
+      </c>
+      <c r="D1202" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="E1202" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1202" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1202" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="H1202" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I1202" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1203" t="n">
+        <v>14</v>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>sa bàn bệnh viện</t>
+        </is>
+      </c>
+      <c r="D1203" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E1203" t="n">
+        <v>590</v>
+      </c>
+      <c r="F1203" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1203" t="inlineStr">
+        <is>
+          <t>4.41%</t>
+        </is>
+      </c>
+      <c r="H1203" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
+        </is>
+      </c>
+      <c r="I1203" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1204" t="n">
+        <v>15</v>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>vận chuyển mô hình</t>
+        </is>
+      </c>
+      <c r="D1204" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E1204" t="n">
+        <v>820</v>
+      </c>
+      <c r="F1204" t="n">
+        <v>45</v>
+      </c>
+      <c r="G1204" t="inlineStr">
+        <is>
+          <t>5.49%</t>
+        </is>
+      </c>
+      <c r="H1204" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1204" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1205" t="n">
+        <v>16</v>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>vận chuyển sa bàn</t>
+        </is>
+      </c>
+      <c r="D1205" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E1205" t="n">
+        <v>760</v>
+      </c>
+      <c r="F1205" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1205" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="H1205" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1205" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1206" t="n">
+        <v>17</v>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>sửa chữa mô hình</t>
+        </is>
+      </c>
+      <c r="D1206" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E1206" t="n">
+        <v>930</v>
+      </c>
+      <c r="F1206" t="n">
+        <v>58</v>
+      </c>
+      <c r="G1206" t="inlineStr">
+        <is>
+          <t>6.24%</t>
+        </is>
+      </c>
+      <c r="H1206" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1206" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1207" t="n">
+        <v>18</v>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>sửa chữa sa bàn</t>
+        </is>
+      </c>
+      <c r="D1207" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E1207" t="n">
+        <v>880</v>
+      </c>
+      <c r="F1207" t="n">
+        <v>52</v>
+      </c>
+      <c r="G1207" t="inlineStr">
+        <is>
+          <t>5.91%</t>
+        </is>
+      </c>
+      <c r="H1207" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1207" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1208" t="n">
+        <v>19</v>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>công ty mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1208" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="E1208" t="n">
+        <v>69</v>
+      </c>
+      <c r="F1208" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1208" t="inlineStr">
+        <is>
+          <t>2.90%</t>
+        </is>
+      </c>
+      <c r="H1208" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="I1208" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1209" t="n">
+        <v>20</v>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>công ty sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1209" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E1209" t="n">
+        <v>2410</v>
+      </c>
+      <c r="F1209" t="n">
+        <v>168</v>
+      </c>
+      <c r="G1209" t="inlineStr">
+        <is>
+          <t>6.97%</t>
+        </is>
+      </c>
+      <c r="H1209" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/</t>
+        </is>
+      </c>
+      <c r="I1209" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1210" t="n">
+        <v>21</v>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>làm mô hình</t>
+        </is>
+      </c>
+      <c r="D1210" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E1210" t="n">
+        <v>1780</v>
+      </c>
+      <c r="F1210" t="n">
+        <v>121</v>
+      </c>
+      <c r="G1210" t="inlineStr">
+        <is>
+          <t>6.80%</t>
+        </is>
+      </c>
+      <c r="H1210" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1210" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B1211" t="n">
+        <v>22</v>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>làm sa bàn</t>
+        </is>
+      </c>
+      <c r="D1211" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E1211" t="n">
+        <v>1620</v>
+      </c>
+      <c r="F1211" t="n">
+        <v>104</v>
+      </c>
+      <c r="G1211" t="inlineStr">
+        <is>
+          <t>6.42%</t>
+        </is>
+      </c>
+      <c r="H1211" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I1211" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1212" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>mô hình quy hoạch</t>
+        </is>
+      </c>
+      <c r="D1212" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="E1212" t="n">
+        <v>82</v>
+      </c>
+      <c r="F1212" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1212" t="inlineStr">
+        <is>
+          <t>8.54%</t>
+        </is>
+      </c>
+      <c r="H1212" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/danh-muc-du-an/mo-hinh-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I1212" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1213" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1213" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="E1213" t="n">
+        <v>343</v>
+      </c>
+      <c r="F1213" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1213" t="inlineStr">
+        <is>
+          <t>2.04%</t>
+        </is>
+      </c>
+      <c r="H1213" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1213" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1214" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>mô hình cao tầng</t>
+        </is>
+      </c>
+      <c r="D1214" t="n">
+        <v>5</v>
+      </c>
+      <c r="E1214" t="n">
+        <v>980</v>
+      </c>
+      <c r="F1214" t="n">
+        <v>54</v>
+      </c>
+      <c r="G1214" t="inlineStr">
+        <is>
+          <t>5.51%</t>
+        </is>
+      </c>
+      <c r="H1214" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I1214" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1215" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>mô hình nhà máy</t>
+        </is>
+      </c>
+      <c r="D1215" t="n">
+        <v>24</v>
+      </c>
+      <c r="E1215" t="n">
+        <v>29</v>
+      </c>
+      <c r="F1215" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1215" t="inlineStr">
+        <is>
+          <t>3.45%</t>
+        </is>
+      </c>
+      <c r="H1215" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-nha-may/</t>
+        </is>
+      </c>
+      <c r="I1215" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1216" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>mô hình thiết bị</t>
+        </is>
+      </c>
+      <c r="D1216" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1216" t="n">
+        <v>640</v>
+      </c>
+      <c r="F1216" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1216" t="inlineStr">
+        <is>
+          <t>3.91%</t>
+        </is>
+      </c>
+      <c r="H1216" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-3d/</t>
+        </is>
+      </c>
+      <c r="I1216" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1217" t="n">
+        <v>6</v>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>mô hình trường học</t>
+        </is>
+      </c>
+      <c r="D1217" t="n">
+        <v>7</v>
+      </c>
+      <c r="E1217" t="n">
+        <v>720</v>
+      </c>
+      <c r="F1217" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1217" t="inlineStr">
+        <is>
+          <t>5.28%</t>
+        </is>
+      </c>
+      <c r="H1217" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I1217" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1218" t="n">
+        <v>7</v>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>mô hình bệnh viện</t>
+        </is>
+      </c>
+      <c r="D1218" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1218" t="n">
+        <v>530</v>
+      </c>
+      <c r="F1218" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1218" t="inlineStr">
+        <is>
+          <t>4.15%</t>
+        </is>
+      </c>
+      <c r="H1218" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/mo-hinh-tod-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I1218" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1219" t="n">
+        <v>8</v>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>sa bàn quy hoạch</t>
+        </is>
+      </c>
+      <c r="D1219" t="n">
+        <v>4</v>
+      </c>
+      <c r="E1219" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F1219" t="n">
+        <v>118</v>
+      </c>
+      <c r="G1219" t="inlineStr">
+        <is>
+          <t>7.15%</t>
+        </is>
+      </c>
+      <c r="H1219" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/dich-vu-lam-sa-ban-quy-hoach/</t>
+        </is>
+      </c>
+      <c r="I1219" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1220" t="n">
+        <v>9</v>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1220" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1220" t="n">
+        <v>44</v>
+      </c>
+      <c r="F1220" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1220" t="inlineStr">
+        <is>
+          <t>2.27%</t>
+        </is>
+      </c>
+      <c r="H1220" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1220" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1221" t="n">
+        <v>10</v>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>sa bàn cao tầng</t>
+        </is>
+      </c>
+      <c r="D1221" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E1221" t="n">
+        <v>870</v>
+      </c>
+      <c r="F1221" t="n">
+        <v>46</v>
+      </c>
+      <c r="G1221" t="inlineStr">
+        <is>
+          <t>5.29%</t>
+        </is>
+      </c>
+      <c r="H1221" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-cao-tang/</t>
+        </is>
+      </c>
+      <c r="I1221" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1222" t="n">
+        <v>11</v>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>sa bàn nhà máy</t>
+        </is>
+      </c>
+      <c r="D1222" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E1222" t="n">
+        <v>30</v>
+      </c>
+      <c r="F1222" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1222" t="inlineStr">
+        <is>
+          <t>3.33%</t>
+        </is>
+      </c>
+      <c r="H1222" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/thi-cong-sa-ban-nha-may-khu-cong-nghiep/</t>
+        </is>
+      </c>
+      <c r="I1222" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1223" t="n">
+        <v>12</v>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>sa bàn thiết bị</t>
+        </is>
+      </c>
+      <c r="D1223" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E1223" t="n">
+        <v>480</v>
+      </c>
+      <c r="F1223" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1223" t="inlineStr">
+        <is>
+          <t>3.75%</t>
+        </is>
+      </c>
+      <c r="H1223" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sa-ban-noi-that/</t>
+        </is>
+      </c>
+      <c r="I1223" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1224" t="n">
+        <v>13</v>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>sa bàn trường học</t>
+        </is>
+      </c>
+      <c r="D1224" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="E1224" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1224" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1224" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="H1224" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban-truong-hoc/</t>
+        </is>
+      </c>
+      <c r="I1224" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1225" t="n">
+        <v>14</v>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>sa bàn bệnh viện</t>
+        </is>
+      </c>
+      <c r="D1225" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E1225" t="n">
+        <v>590</v>
+      </c>
+      <c r="F1225" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1225" t="inlineStr">
+        <is>
+          <t>4.41%</t>
+        </is>
+      </c>
+      <c r="H1225" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/du-an-noi-bat/</t>
+        </is>
+      </c>
+      <c r="I1225" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1226" t="n">
+        <v>15</v>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>vận chuyển mô hình</t>
+        </is>
+      </c>
+      <c r="D1226" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E1226" t="n">
+        <v>820</v>
+      </c>
+      <c r="F1226" t="n">
+        <v>45</v>
+      </c>
+      <c r="G1226" t="inlineStr">
+        <is>
+          <t>5.49%</t>
+        </is>
+      </c>
+      <c r="H1226" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1226" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1227" t="n">
+        <v>16</v>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>vận chuyển sa bàn</t>
+        </is>
+      </c>
+      <c r="D1227" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E1227" t="n">
+        <v>760</v>
+      </c>
+      <c r="F1227" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1227" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="H1227" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/van-chuyen-sa-ban-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1227" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1228" t="n">
+        <v>17</v>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>sửa chữa mô hình</t>
+        </is>
+      </c>
+      <c r="D1228" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E1228" t="n">
+        <v>930</v>
+      </c>
+      <c r="F1228" t="n">
+        <v>58</v>
+      </c>
+      <c r="G1228" t="inlineStr">
+        <is>
+          <t>6.24%</t>
+        </is>
+      </c>
+      <c r="H1228" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1228" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1229" t="n">
+        <v>18</v>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>sửa chữa sa bàn</t>
+        </is>
+      </c>
+      <c r="D1229" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E1229" t="n">
+        <v>880</v>
+      </c>
+      <c r="F1229" t="n">
+        <v>52</v>
+      </c>
+      <c r="G1229" t="inlineStr">
+        <is>
+          <t>5.91%</t>
+        </is>
+      </c>
+      <c r="H1229" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/sua-chua-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1229" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1230" t="n">
+        <v>19</v>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>công ty mô hình kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1230" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="E1230" t="n">
+        <v>69</v>
+      </c>
+      <c r="F1230" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1230" t="inlineStr">
+        <is>
+          <t>2.90%</t>
+        </is>
+      </c>
+      <c r="H1230" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/cong-ty-lam-mo-hinh/</t>
+        </is>
+      </c>
+      <c r="I1230" t="inlineStr">
+        <is>
+          <t>🖼️ Image Pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1231" t="n">
+        <v>20</v>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>công ty sa bàn kiến trúc</t>
+        </is>
+      </c>
+      <c r="D1231" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E1231" t="n">
+        <v>2410</v>
+      </c>
+      <c r="F1231" t="n">
+        <v>168</v>
+      </c>
+      <c r="G1231" t="inlineStr">
+        <is>
+          <t>6.97%</t>
+        </is>
+      </c>
+      <c r="H1231" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/</t>
+        </is>
+      </c>
+      <c r="I1231" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1232" t="n">
+        <v>21</v>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>làm mô hình</t>
+        </is>
+      </c>
+      <c r="D1232" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E1232" t="n">
+        <v>1780</v>
+      </c>
+      <c r="F1232" t="n">
+        <v>121</v>
+      </c>
+      <c r="G1232" t="inlineStr">
+        <is>
+          <t>6.80%</t>
+        </is>
+      </c>
+      <c r="H1232" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-mo-hinh-kien-truc/</t>
+        </is>
+      </c>
+      <c r="I1232" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B1233" t="n">
+        <v>22</v>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>làm sa bàn</t>
+        </is>
+      </c>
+      <c r="D1233" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E1233" t="n">
+        <v>1620</v>
+      </c>
+      <c r="F1233" t="n">
+        <v>104</v>
+      </c>
+      <c r="G1233" t="inlineStr">
+        <is>
+          <t>6.42%</t>
+        </is>
+      </c>
+      <c r="H1233" t="inlineStr">
+        <is>
+          <t>https://mohinhkientruc.org/lam-sa-ban/</t>
+        </is>
+      </c>
+      <c r="I1233" t="inlineStr">
+        <is>
+          <t>Standard Snippet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>